<commit_message>
reformat Betas params for Gina
</commit_message>
<xml_diff>
--- a/data/raw/Betas params for Gina.xlsx
+++ b/data/raw/Betas params for Gina.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\awl.IC\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au757887\PC_documents\_git-it\PPATonline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{088215D3-B557-4490-A3B1-F069A2278B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98DF5459-4680-4D6A-89AE-197836C1B1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{5E83B20B-DA4B-4D40-A213-CF41A4D2295F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E83B20B-DA4B-4D40-A213-CF41A4D2295F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -644,288 +644,288 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D44B70B-6ED1-4DFA-81D1-A0B0F4EF83B6}">
-  <dimension ref="C5:I17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="5" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="7">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="8">
+        <v>1.1532748734247142</v>
+      </c>
+      <c r="E3" s="8">
+        <v>1.4141182843558209</v>
+      </c>
+      <c r="F3" s="8">
+        <v>2.7943942098127432</v>
+      </c>
+      <c r="G3" s="8">
+        <v>4.1384732454790258</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1.8635022610226373</v>
+      </c>
+      <c r="E4" s="10">
+        <v>3.3986974761189108</v>
+      </c>
+      <c r="F4" s="10">
+        <v>10.778940534936554</v>
+      </c>
+      <c r="G4" s="10">
+        <v>17.452284257064413</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
       <c r="C5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="3:9" ht="30.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="10">
+        <v>2.7588973578217617</v>
+      </c>
+      <c r="E5" s="10">
+        <v>5.8157820283280657</v>
+      </c>
+      <c r="F5" s="10">
+        <v>20.363937977742658</v>
+      </c>
+      <c r="G5" s="10">
+        <v>33.386675853198597</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8">
-        <v>1.1532748734247142</v>
-      </c>
-      <c r="G7" s="8">
-        <v>1.4141182843558209</v>
-      </c>
-      <c r="H7" s="8">
-        <v>2.7943942098127432</v>
-      </c>
-      <c r="I7" s="8">
-        <v>4.1384732454790258</v>
-      </c>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="10">
-        <v>1.8635022610226373</v>
-      </c>
-      <c r="G8" s="10">
-        <v>3.3986974761189108</v>
-      </c>
-      <c r="H8" s="10">
-        <v>10.778940534936554</v>
-      </c>
-      <c r="I8" s="10">
-        <v>17.452284257064413</v>
-      </c>
-    </row>
-    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C9" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="10">
-        <v>2.7588973578217617</v>
-      </c>
-      <c r="G9" s="10">
-        <v>5.8157820283280657</v>
-      </c>
-      <c r="H9" s="10">
-        <v>20.363937977742658</v>
-      </c>
-      <c r="I9" s="10">
-        <v>33.386675853198597</v>
-      </c>
-    </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10">
-        <v>4</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="11">
-        <f t="shared" ref="F10:H10" si="0">F13</f>
+      <c r="D6" s="11">
+        <f t="shared" ref="D6:F6" si="0">D9</f>
         <v>3.0148386090528208</v>
       </c>
-      <c r="G10" s="11">
+      <c r="E6" s="11">
         <f t="shared" si="0"/>
         <v>6.5969607776107919</v>
       </c>
-      <c r="H10" s="11">
+      <c r="F6" s="11">
         <f t="shared" si="0"/>
         <v>23.817527914851958</v>
       </c>
-      <c r="I10" s="11">
-        <f>I13</f>
+      <c r="G6" s="11">
+        <f>G9</f>
         <v>39.388663266483633</v>
       </c>
     </row>
-    <row r="11" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="9" t="s">
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D11">
+      <c r="B7">
         <v>5</v>
       </c>
-      <c r="E11" t="s">
+      <c r="C7" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="11">
-        <f t="shared" ref="F11:H11" si="1">F12</f>
+      <c r="D7" s="11">
+        <f t="shared" ref="D7:F7" si="1">D8</f>
         <v>2.379473860822428</v>
       </c>
-      <c r="G11" s="11">
+      <c r="E7" s="11">
         <f t="shared" si="1"/>
         <v>4.7270645592023879</v>
       </c>
-      <c r="H11" s="11">
+      <c r="F7" s="11">
         <f t="shared" si="1"/>
         <v>17.149547888314689</v>
       </c>
-      <c r="I11" s="11">
-        <f>I12</f>
+      <c r="G7" s="11">
+        <f>G8</f>
         <v>29.24625920931123</v>
       </c>
     </row>
-    <row r="12" spans="3:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="12" t="s">
+    <row r="8" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="13">
+      <c r="B8" s="13">
         <v>1</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="C8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="14">
+      <c r="D8" s="14">
         <v>2.379473860822428</v>
       </c>
-      <c r="G12" s="14">
+      <c r="E8" s="14">
         <v>4.7270645592023879</v>
       </c>
-      <c r="H12" s="14">
+      <c r="F8" s="14">
         <v>17.149547888314689</v>
       </c>
-      <c r="I12" s="14">
+      <c r="G8" s="14">
         <v>29.24625920931123</v>
       </c>
     </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="9" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D13">
+      <c r="B9">
         <v>2</v>
       </c>
-      <c r="E13" t="s">
+      <c r="C9" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="10">
+      <c r="D9" s="10">
         <v>3.0148386090528208</v>
       </c>
-      <c r="G13" s="10">
+      <c r="E9" s="10">
         <v>6.5969607776107919</v>
       </c>
-      <c r="H13" s="10">
+      <c r="F9" s="10">
         <v>23.817527914851958</v>
       </c>
-      <c r="I13" s="10">
+      <c r="G9" s="10">
         <v>39.388663266483633</v>
       </c>
     </row>
-    <row r="14" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C14" s="9" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D14">
+      <c r="B10">
         <v>3</v>
       </c>
-      <c r="E14" t="s">
+      <c r="C10" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="15">
-        <f>F9</f>
+      <c r="D10" s="15">
+        <f>D5</f>
         <v>2.7588973578217617</v>
       </c>
-      <c r="G14" s="15">
-        <f>G9</f>
+      <c r="E10" s="15">
+        <f>E5</f>
         <v>5.8157820283280657</v>
       </c>
-      <c r="H14" s="15">
-        <f>H9</f>
+      <c r="F10" s="15">
+        <f>F5</f>
         <v>20.363937977742658</v>
       </c>
-      <c r="I14" s="15">
-        <f>I9</f>
+      <c r="G10" s="15">
+        <f>G5</f>
         <v>33.386675853198597</v>
       </c>
     </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="9" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D15">
+      <c r="B11">
         <v>4</v>
       </c>
-      <c r="E15" t="s">
+      <c r="C11" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="11">
-        <f>F8</f>
+      <c r="D11" s="11">
+        <f>D4</f>
         <v>1.8635022610226373</v>
       </c>
-      <c r="G15" s="11">
-        <f>G8</f>
+      <c r="E11" s="11">
+        <f>E4</f>
         <v>3.3986974761189108</v>
       </c>
-      <c r="H15" s="11">
-        <f>H8</f>
+      <c r="F11" s="11">
+        <f>F4</f>
         <v>10.778940534936554</v>
       </c>
-      <c r="I15" s="11">
-        <f>I8</f>
+      <c r="G11" s="11">
+        <f>G4</f>
         <v>17.452284257064413</v>
       </c>
     </row>
-    <row r="16" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="16" t="s">
+    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="17">
+      <c r="B12" s="17">
         <v>5</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="C12" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="18">
-        <f>F7</f>
+      <c r="D12" s="18">
+        <f>D3</f>
         <v>1.1532748734247142</v>
       </c>
-      <c r="G16" s="18">
-        <f>G7</f>
+      <c r="E12" s="18">
+        <f>E3</f>
         <v>1.4141182843558209</v>
       </c>
-      <c r="H16" s="18">
-        <f>H7</f>
+      <c r="F12" s="18">
+        <f>F3</f>
         <v>2.7943942098127432</v>
       </c>
-      <c r="I16" s="18">
-        <f>I7</f>
+      <c r="G12" s="18">
+        <f>G3</f>
         <v>4.1384732454790258</v>
       </c>
     </row>
-    <row r="17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>